<commit_message>
Update dashboard market share
</commit_message>
<xml_diff>
--- a/FB Market Share.xlsx
+++ b/FB Market Share.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6350"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6350" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="KEC MS MOM " sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="665" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="671" uniqueCount="97">
   <si>
     <t>LMTD</t>
   </si>
@@ -303,6 +303,18 @@
   <si>
     <t>NAMA PT</t>
   </si>
+  <si>
+    <t>W4-Jul</t>
+  </si>
+  <si>
+    <t>W4-Aug</t>
+  </si>
+  <si>
+    <t>W5-Aug</t>
+  </si>
+  <si>
+    <t>WoW</t>
+  </si>
 </sst>
 </file>
 
@@ -312,7 +324,7 @@
     <numFmt numFmtId="164" formatCode="mmm\-d"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -395,8 +407,21 @@
       <name val="Century Gothic"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Century Gothic"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color indexed="8"/>
+      <name val="Century Gothic"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -487,6 +512,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FF595959"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -536,7 +567,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -678,6 +709,19 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="15" fillId="15" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="15" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1103,97 +1147,97 @@
       <c r="O3" s="4"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
-      <c r="R3" s="51" t="s">
+      <c r="R3" s="56" t="s">
         <v>11</v>
       </c>
-      <c r="S3" s="52"/>
-      <c r="T3" s="52"/>
-      <c r="U3" s="52"/>
-      <c r="V3" s="52"/>
-      <c r="W3" s="52"/>
-      <c r="X3" s="52"/>
-      <c r="Y3" s="52"/>
-      <c r="Z3" s="52"/>
-      <c r="AA3" s="52"/>
-      <c r="AB3" s="52"/>
-      <c r="AC3" s="51" t="s">
+      <c r="S3" s="57"/>
+      <c r="T3" s="57"/>
+      <c r="U3" s="57"/>
+      <c r="V3" s="57"/>
+      <c r="W3" s="57"/>
+      <c r="X3" s="57"/>
+      <c r="Y3" s="57"/>
+      <c r="Z3" s="57"/>
+      <c r="AA3" s="57"/>
+      <c r="AB3" s="57"/>
+      <c r="AC3" s="56" t="s">
         <v>4</v>
       </c>
-      <c r="AD3" s="52"/>
-      <c r="AE3" s="52"/>
-      <c r="AF3" s="52"/>
-      <c r="AG3" s="52"/>
-      <c r="AH3" s="52"/>
-      <c r="AI3" s="52"/>
-      <c r="AJ3" s="52"/>
-      <c r="AK3" s="52"/>
-      <c r="AL3" s="52"/>
-      <c r="AM3" s="52"/>
-      <c r="AN3" s="51" t="s">
+      <c r="AD3" s="57"/>
+      <c r="AE3" s="57"/>
+      <c r="AF3" s="57"/>
+      <c r="AG3" s="57"/>
+      <c r="AH3" s="57"/>
+      <c r="AI3" s="57"/>
+      <c r="AJ3" s="57"/>
+      <c r="AK3" s="57"/>
+      <c r="AL3" s="57"/>
+      <c r="AM3" s="57"/>
+      <c r="AN3" s="56" t="s">
         <v>5</v>
       </c>
-      <c r="AO3" s="52"/>
-      <c r="AP3" s="52"/>
-      <c r="AQ3" s="52"/>
-      <c r="AR3" s="52"/>
-      <c r="AS3" s="52"/>
-      <c r="AT3" s="52"/>
-      <c r="AU3" s="52"/>
-      <c r="AV3" s="52"/>
-      <c r="AW3" s="52"/>
-      <c r="AX3" s="52"/>
-      <c r="AY3" s="51" t="s">
+      <c r="AO3" s="57"/>
+      <c r="AP3" s="57"/>
+      <c r="AQ3" s="57"/>
+      <c r="AR3" s="57"/>
+      <c r="AS3" s="57"/>
+      <c r="AT3" s="57"/>
+      <c r="AU3" s="57"/>
+      <c r="AV3" s="57"/>
+      <c r="AW3" s="57"/>
+      <c r="AX3" s="57"/>
+      <c r="AY3" s="56" t="s">
         <v>6</v>
       </c>
-      <c r="AZ3" s="52"/>
-      <c r="BA3" s="52"/>
-      <c r="BB3" s="52"/>
-      <c r="BC3" s="52"/>
-      <c r="BD3" s="52"/>
-      <c r="BE3" s="52"/>
-      <c r="BF3" s="52"/>
-      <c r="BG3" s="52"/>
-      <c r="BH3" s="52"/>
-      <c r="BI3" s="52"/>
-      <c r="BJ3" s="51" t="s">
+      <c r="AZ3" s="57"/>
+      <c r="BA3" s="57"/>
+      <c r="BB3" s="57"/>
+      <c r="BC3" s="57"/>
+      <c r="BD3" s="57"/>
+      <c r="BE3" s="57"/>
+      <c r="BF3" s="57"/>
+      <c r="BG3" s="57"/>
+      <c r="BH3" s="57"/>
+      <c r="BI3" s="57"/>
+      <c r="BJ3" s="56" t="s">
         <v>7</v>
       </c>
-      <c r="BK3" s="52"/>
-      <c r="BL3" s="52"/>
-      <c r="BM3" s="52"/>
-      <c r="BN3" s="52"/>
-      <c r="BO3" s="52"/>
-      <c r="BP3" s="52"/>
-      <c r="BQ3" s="52"/>
-      <c r="BR3" s="52"/>
-      <c r="BS3" s="52"/>
-      <c r="BT3" s="52"/>
-      <c r="BU3" s="51" t="s">
+      <c r="BK3" s="57"/>
+      <c r="BL3" s="57"/>
+      <c r="BM3" s="57"/>
+      <c r="BN3" s="57"/>
+      <c r="BO3" s="57"/>
+      <c r="BP3" s="57"/>
+      <c r="BQ3" s="57"/>
+      <c r="BR3" s="57"/>
+      <c r="BS3" s="57"/>
+      <c r="BT3" s="57"/>
+      <c r="BU3" s="56" t="s">
         <v>8</v>
       </c>
-      <c r="BV3" s="52"/>
-      <c r="BW3" s="52"/>
-      <c r="BX3" s="52"/>
-      <c r="BY3" s="52"/>
-      <c r="BZ3" s="52"/>
-      <c r="CA3" s="52"/>
-      <c r="CB3" s="52"/>
-      <c r="CC3" s="52"/>
-      <c r="CD3" s="52"/>
-      <c r="CE3" s="52"/>
-      <c r="CF3" s="51" t="s">
+      <c r="BV3" s="57"/>
+      <c r="BW3" s="57"/>
+      <c r="BX3" s="57"/>
+      <c r="BY3" s="57"/>
+      <c r="BZ3" s="57"/>
+      <c r="CA3" s="57"/>
+      <c r="CB3" s="57"/>
+      <c r="CC3" s="57"/>
+      <c r="CD3" s="57"/>
+      <c r="CE3" s="57"/>
+      <c r="CF3" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="CG3" s="52"/>
-      <c r="CH3" s="52"/>
-      <c r="CI3" s="52"/>
-      <c r="CJ3" s="52"/>
-      <c r="CK3" s="52"/>
-      <c r="CL3" s="52"/>
-      <c r="CM3" s="52"/>
-      <c r="CN3" s="52"/>
-      <c r="CO3" s="52"/>
-      <c r="CP3" s="52"/>
+      <c r="CG3" s="57"/>
+      <c r="CH3" s="57"/>
+      <c r="CI3" s="57"/>
+      <c r="CJ3" s="57"/>
+      <c r="CK3" s="57"/>
+      <c r="CL3" s="57"/>
+      <c r="CM3" s="57"/>
+      <c r="CN3" s="57"/>
+      <c r="CO3" s="57"/>
+      <c r="CP3" s="57"/>
     </row>
     <row r="4" spans="1:94" ht="15" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
@@ -6406,35 +6450,24 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A2:S4"/>
+  <dimension ref="A2:Y4"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="19" width="12.453125" customWidth="1"/>
+    <col min="2" max="7" width="25.08984375" style="51" customWidth="1"/>
+    <col min="8" max="25" width="12.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:19" ht="15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:25" ht="15" x14ac:dyDescent="0.3">
       <c r="A2" s="42">
         <v>46264</v>
       </c>
-      <c r="B2" s="29" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="29" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="29" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" s="29" t="s">
-        <v>0</v>
-      </c>
-      <c r="F2" s="29" t="s">
-        <v>1</v>
-      </c>
-      <c r="G2" s="29" t="s">
-        <v>2</v>
-      </c>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
       <c r="H2" s="29" t="s">
         <v>0</v>
       </c>
@@ -6450,149 +6483,204 @@
       <c r="L2" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="M2" s="30" t="s">
+      <c r="M2" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="N2" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="O2" s="30" t="s">
+      <c r="N2" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="O2" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="P2" s="30" t="s">
+      <c r="P2" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="Q2" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="R2" s="30" t="s">
+      <c r="Q2" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="R2" s="29" t="s">
         <v>1</v>
       </c>
       <c r="S2" s="30" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:19" ht="15" x14ac:dyDescent="0.3">
+      <c r="T2" s="30" t="s">
+        <v>0</v>
+      </c>
+      <c r="U2" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="V2" s="30" t="s">
+        <v>2</v>
+      </c>
+      <c r="W2" s="30" t="s">
+        <v>0</v>
+      </c>
+      <c r="X2" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y2" s="30" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25" ht="15" x14ac:dyDescent="0.3">
       <c r="A3" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="53" t="s">
+        <v>93</v>
+      </c>
+      <c r="C3" s="53" t="s">
+        <v>39</v>
+      </c>
+      <c r="D3" s="53" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" s="53" t="s">
+        <v>94</v>
+      </c>
+      <c r="F3" s="53" t="s">
+        <v>95</v>
+      </c>
+      <c r="G3" s="53" t="s">
+        <v>96</v>
+      </c>
+      <c r="H3" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="32" t="s">
+      <c r="I3" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="32" t="s">
+      <c r="J3" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="33" t="s">
+      <c r="K3" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="33" t="s">
+      <c r="L3" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="33" t="s">
+      <c r="M3" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="34" t="s">
+      <c r="N3" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="I3" s="34" t="s">
+      <c r="O3" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="J3" s="34" t="s">
+      <c r="P3" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="K3" s="35" t="s">
+      <c r="Q3" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="L3" s="35" t="s">
+      <c r="R3" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="M3" s="36" t="s">
+      <c r="S3" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="N3" s="37" t="s">
+      <c r="T3" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="O3" s="37" t="s">
+      <c r="U3" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="P3" s="37" t="s">
+      <c r="V3" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="Q3" s="38" t="s">
+      <c r="W3" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="R3" s="38" t="s">
+      <c r="X3" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="S3" s="38" t="s">
+      <c r="Y3" s="38" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="40">
+      <c r="B4" s="54">
         <v>0.343542430432489</v>
       </c>
-      <c r="C4" s="40">
+      <c r="C4" s="54">
+        <v>0.33758422899148</v>
+      </c>
+      <c r="D4" s="54">
+        <v>0.339650831985919</v>
+      </c>
+      <c r="E4" s="54">
+        <v>0.33818616907233601</v>
+      </c>
+      <c r="F4" s="54">
         <v>0.33675168049224202</v>
       </c>
-      <c r="D4" s="41">
-        <f>IFERROR(C4-B4,"")</f>
-        <v>-6.7907499402469762E-3</v>
-      </c>
-      <c r="E4" s="40">
-        <v>8.7694971658933196E-2</v>
-      </c>
-      <c r="F4" s="40">
-        <v>8.8678012769633802E-2</v>
-      </c>
-      <c r="G4" s="41">
-        <f>IFERROR(F4-E4,"")</f>
-        <v>9.830411107006054E-4</v>
+      <c r="G4" s="55">
+        <f>F4-E4</f>
+        <v>-1.4344885800939844E-3</v>
       </c>
       <c r="H4" s="40">
-        <v>0.39116083386317801</v>
+        <v>0.343542430432489</v>
       </c>
       <c r="I4" s="40">
-        <v>0.38795664786575701</v>
+        <v>0.33675168049224202</v>
       </c>
       <c r="J4" s="41">
         <f>IFERROR(I4-H4,"")</f>
-        <v>-3.2041859974210052E-3</v>
+        <v>-6.7907499402469762E-3</v>
       </c>
       <c r="K4" s="40">
-        <v>0.17760176404540001</v>
+        <v>8.7694971658933196E-2</v>
       </c>
       <c r="L4" s="40">
-        <v>0.186613658872367</v>
+        <v>8.8678012769633802E-2</v>
       </c>
       <c r="M4" s="41">
         <f>IFERROR(L4-K4,"")</f>
-        <v>9.0118948269669874E-3</v>
+        <v>9.830411107006054E-4</v>
       </c>
       <c r="N4" s="40">
-        <v>0.166860567362455</v>
+        <v>0.39116083386317801</v>
       </c>
       <c r="O4" s="40">
-        <v>0.17595824933798801</v>
+        <v>0.38795664786575701</v>
       </c>
       <c r="P4" s="41">
         <f>IFERROR(O4-N4,"")</f>
-        <v>9.0976819755330118E-3</v>
+        <v>-3.2041859974210052E-3</v>
       </c>
       <c r="Q4" s="40">
-        <v>1.0741196682945301E-2</v>
+        <v>0.17760176404540001</v>
       </c>
       <c r="R4" s="40">
-        <v>1.0655409534379E-2</v>
+        <v>0.186613658872367</v>
       </c>
       <c r="S4" s="41">
         <f>IFERROR(R4-Q4,"")</f>
+        <v>9.0118948269669874E-3</v>
+      </c>
+      <c r="T4" s="40">
+        <v>0.166860567362455</v>
+      </c>
+      <c r="U4" s="40">
+        <v>0.17595824933798801</v>
+      </c>
+      <c r="V4" s="41">
+        <f>IFERROR(U4-T4,"")</f>
+        <v>9.0976819755330118E-3</v>
+      </c>
+      <c r="W4" s="40">
+        <v>1.0741196682945301E-2</v>
+      </c>
+      <c r="X4" s="40">
+        <v>1.0655409534379E-2</v>
+      </c>
+      <c r="Y4" s="41">
+        <f>IFERROR(X4-W4,"")</f>
         <v>-8.578714856630025E-5</v>
       </c>
     </row>

</xml_diff>